<commit_message>
Add illustrative Upside Case (Y3) sheet to the financial model
New tab shows a Year 3 P&L/cash-flow scenario for the 5-hire
job-creation target (6 paying universities, 1,500 premium
subscribers), reconciled against the same methodology as the
existing base-case sheets. Ends the year at +£6,770 cash, no
external funding needed. Clearly labelled illustrative/founder-
prepared, not part of the core conservative 3-year forecast.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/visa_appendices/DEQUAD_Financial_Model.xlsx
+++ b/visa_appendices/DEQUAD_Financial_Model.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="P&amp;L 3yr" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Cash Flow 3yr" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flow Y1 (mo)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Balance Sheet 3yr" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Revenue W1" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Cost of Sales W2" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Payroll W3" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Marketing W4" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="R&amp;D W5" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Fixed Assets" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Accelerator Value" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Startup Loan" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P&amp;L 3yr" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow 3yr" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow Y1 (mo)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet 3yr" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue W1" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost of Sales W2" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payroll W3" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing W4" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R&amp;D W5" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixed Assets" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accelerator Value" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startup Loan" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upside Case (Y3)" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,10 +29,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="£#,##0;[Red](£#,##0);&quot;-&quot;"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,6 +76,26 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000F2942"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="004F6076"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000F2942"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -125,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -171,6 +194,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -536,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A48"/>
+  <dimension ref="A1:A51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -717,146 +754,167 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Office, legal and accountancy carry a nominal £0 cash cost in Y1 because</t>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - See the "Upside Case (Y3)" sheet for the job-creation-target scenario (5 full-time</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    those services are provided FREE by the NatWest Accelerator (Y1 only).</t>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    hires, avg £25,000/yr, meeting the Innovator Founder settlement job-creation criterion).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Marketing is founder-led and low-cost throughout — no paid-acquisition</t>
+          <t xml:space="preserve">  - Office, legal and accountancy carry a nominal £0 cash cost in Y1 because</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">    budget in Y1; spend grows only in line with actual revenue in Y2-Y3.</t>
+          <t xml:space="preserve">    those services are provided FREE by the NatWest Accelerator (Y1 only).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Marketing is founder-led and low-cost throughout — no paid-acquisition</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    budget in Y1; spend grows only in line with actual revenue in Y2-Y3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Y1 starts with the existing MVP, so no upfront engineering capex.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>WORKBOOK STRUCTURE</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1. P&amp;L 3yr            — Annual Profit &amp; Loss</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2. Cash Flow 3yr      — Annual cash flow forecast</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3. Cash Flow Y1 (mo)  — Monthly cash flow for Year 1</t>
+          <t xml:space="preserve">  1. P&amp;L 3yr            — Annual Profit &amp; Loss</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  4. Balance Sheet 3yr  — Year-end balance sheets</t>
+          <t xml:space="preserve">  2. Cash Flow 3yr      — Annual cash flow forecast</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  5. Revenue W1         — Revenue detail by service</t>
+          <t xml:space="preserve">  3. Cash Flow Y1 (mo)  — Monthly cash flow for Year 1</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  6. Cost of Sales W2   — Direct cost detail</t>
+          <t xml:space="preserve">  4. Balance Sheet 3yr  — Year-end balance sheets</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  7. Payroll W3         — Salaries, NI and pension</t>
+          <t xml:space="preserve">  5. Revenue W1         — Revenue detail by service</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  8. Marketing W4       — Marketing spend by channel</t>
+          <t xml:space="preserve">  6. Cost of Sales W2   — Direct cost detail</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  9. R&amp;D W5             — R&amp;D activity (unpaid founder time; no tax credit assumed)</t>
+          <t xml:space="preserve">  7. Payroll W3         — Salaries, NI and pension</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 10. Fixed Assets       — CAPEX schedule</t>
+          <t xml:space="preserve">  8. Marketing W4       — Marketing spend by channel</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 11. Accelerator Value  — Quantified in-kind value of NatWest support (Y1 only)</t>
+          <t xml:space="preserve">  9. R&amp;D W5             — R&amp;D activity (unpaid founder time; no tax credit assumed)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 12. Startup Loan       — Empty (no debt taken; no external funding assumed at all)</t>
+          <t xml:space="preserve"> 10. Fixed Assets       — CAPEX schedule</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr"/>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 11. Accelerator Value  — Quantified in-kind value of NatWest support (Y1 only)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve"> 12. Startup Loan       — Empty (no debt taken; no external funding assumed at all)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 13. Upside Case (Y3)  — Illustrative Y3 P&amp;L for the 5-hire job-creation target</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
           <t>All assumptions map to DEQUAD_UKES_Business_Plan.md (v5.0, self-funded revision).</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>Yellow cells indicate user-editable inputs.</t>
         </is>
@@ -1420,6 +1478,629 @@
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A6:E6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>Upside Case — Job-Creation Target (Year 3 only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>ILLUSTRATIVE — not part of the core 3-year self-funded forecast (see P&amp;L 3yr / Payroll W3). This scenario shows what Year 3 would look like if institutional revenue scales beyond the conservative base case via pilot conversion (5+ paying universities), funding the plan's job-creation target of 5 full-time UK hires (Student Ambassador, Social Media Manager, Marketing Intern, Sales Lead, Support Agent — Appendix G), each sustained 12+ months at an average salary of £25,000/year, meeting the Innovator Founder settlement job-creation criterion. Years 1-2 are identical to the base case (no institutional revenue is assumed until pilot conversion). Figures are a founder-prepared illustrative projection, not a commitment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="21" t="n"/>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>Y3 Base Case</t>
+        </is>
+      </c>
+      <c r="C4" s="22" t="inlineStr">
+        <is>
+          <t>Y3 Upside Case</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="n"/>
+      <c r="C5" s="24" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Institutional (universities, £20,000/yr each)</t>
+        </is>
+      </c>
+      <c r="B6" s="25" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C6" s="25" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Institutional — university count (avg in year)</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C7" s="26" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Premium (DEQUAD Premium, £59.88/yr avg)</t>
+        </is>
+      </c>
+      <c r="B8" s="25" t="n">
+        <v>18000</v>
+      </c>
+      <c r="C8" s="25" t="n">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Premium — avg subscribers</t>
+        </is>
+      </c>
+      <c r="B9" s="27" t="n">
+        <v>300</v>
+      </c>
+      <c r="C9" s="27" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="28" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="n">
+        <v>48000</v>
+      </c>
+      <c r="C10" s="29" t="n">
+        <v>210000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>Cost of Sales</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="n"/>
+      <c r="C12" s="24" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Cloud hosting (Render, Cloudflare)</t>
+        </is>
+      </c>
+      <c r="B13" s="25" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C13" s="25" t="n">
+        <v>9600</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>LLM / safeguarding inference</t>
+        </is>
+      </c>
+      <c r="B14" s="25" t="n">
+        <v>1800</v>
+      </c>
+      <c r="C14" s="25" t="n">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Stripe processing</t>
+        </is>
+      </c>
+      <c r="B15" s="25" t="n">
+        <v>180</v>
+      </c>
+      <c r="C15" s="25" t="n">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SMS &amp; email (Twilio, SendGrid)</t>
+        </is>
+      </c>
+      <c r="B16" s="25" t="n">
+        <v>800</v>
+      </c>
+      <c r="C16" s="25" t="n">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Customer-success tooling</t>
+        </is>
+      </c>
+      <c r="B17" s="25" t="n">
+        <v>920</v>
+      </c>
+      <c r="C17" s="25" t="n">
+        <v>3700</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="28" t="inlineStr">
+        <is>
+          <t>Total Cost of Sales</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="n">
+        <v>6100</v>
+      </c>
+      <c r="C18" s="29" t="n">
+        <v>24600</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="28" t="inlineStr">
+        <is>
+          <t>Gross Profit / (Loss)</t>
+        </is>
+      </c>
+      <c r="B20" s="29" t="n">
+        <v>41900</v>
+      </c>
+      <c r="C20" s="29" t="n">
+        <v>185400</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Gross margin %</t>
+        </is>
+      </c>
+      <c r="B21" s="30" t="n">
+        <v>0.873</v>
+      </c>
+      <c r="C21" s="30" t="n">
+        <v>0.883</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>Payroll (Year 3)</t>
+        </is>
+      </c>
+      <c r="B23" s="24" t="n"/>
+      <c r="C23" s="24" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Founder A — CEO, £500/mo</t>
+        </is>
+      </c>
+      <c r="B24" s="25" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C24" s="25" t="n">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Founder B — CTO, £500/mo</t>
+        </is>
+      </c>
+      <c r="B25" s="25" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C25" s="25" t="n">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Safeguarding &amp; Trust Lead (part-time) — base case only</t>
+        </is>
+      </c>
+      <c r="B26" s="25" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C26" s="25" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Student Ambassador — full-time, £25,000/yr</t>
+        </is>
+      </c>
+      <c r="B27" s="25" t="n"/>
+      <c r="C27" s="25" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Social Media Manager — full-time, £25,000/yr</t>
+        </is>
+      </c>
+      <c r="B28" s="25" t="n"/>
+      <c r="C28" s="25" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Marketing Intern — full-time, £25,000/yr</t>
+        </is>
+      </c>
+      <c r="B29" s="25" t="n"/>
+      <c r="C29" s="25" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Sales Lead — full-time, £25,000/yr</t>
+        </is>
+      </c>
+      <c r="B30" s="25" t="n"/>
+      <c r="C30" s="25" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Support Agent — full-time, £25,000/yr</t>
+        </is>
+      </c>
+      <c r="B31" s="25" t="n"/>
+      <c r="C31" s="25" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Total gross salaries</t>
+        </is>
+      </c>
+      <c r="B32" s="25" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C32" s="25" t="n">
+        <v>137000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Employer NI (13.8% above secondary threshold)</t>
+        </is>
+      </c>
+      <c r="B33" s="25" t="n">
+        <v>900</v>
+      </c>
+      <c r="C33" s="25" t="n">
+        <v>11000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Employer pension (3% above £6,240)</t>
+        </is>
+      </c>
+      <c r="B34" s="25" t="n">
+        <v>350</v>
+      </c>
+      <c r="C34" s="25" t="n">
+        <v>2800</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Other employment costs (kit, onboarding, training)</t>
+        </is>
+      </c>
+      <c r="B35" s="25" t="n">
+        <v>250</v>
+      </c>
+      <c r="C35" s="25" t="n">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="28" t="inlineStr">
+        <is>
+          <t>Total Employment Cost</t>
+        </is>
+      </c>
+      <c r="B36" s="29" t="n">
+        <v>21500</v>
+      </c>
+      <c r="C36" s="29" t="n">
+        <v>152050</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="23" t="inlineStr">
+        <is>
+          <t>Other Operating Expenses</t>
+        </is>
+      </c>
+      <c r="B38" s="24" t="n"/>
+      <c r="C38" s="24" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Marketing (paid channels, campaigns)</t>
+        </is>
+      </c>
+      <c r="B39" s="25" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C39" s="25" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Software subscriptions (incl. CRM, helpdesk)</t>
+        </is>
+      </c>
+      <c r="B40" s="25" t="n">
+        <v>1800</v>
+      </c>
+      <c r="C40" s="25" t="n">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Office / co-working (7 people vs 3)</t>
+        </is>
+      </c>
+      <c r="B41" s="25" t="n">
+        <v>600</v>
+      </c>
+      <c r="C41" s="25" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Legal &amp; accountancy</t>
+        </is>
+      </c>
+      <c r="B42" s="25" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C42" s="25" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Insurance (D&amp;O, PI, Cyber, EL)</t>
+        </is>
+      </c>
+      <c r="B43" s="25" t="n">
+        <v>900</v>
+      </c>
+      <c r="C43" s="25" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Business support / misc</t>
+        </is>
+      </c>
+      <c r="B44" s="25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C44" s="25" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Fixed assets capex (kit for new hires)</t>
+        </is>
+      </c>
+      <c r="B45" s="25" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C45" s="25" t="n">
+        <v>2800</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="28" t="inlineStr">
+        <is>
+          <t>Total Other OPEX</t>
+        </is>
+      </c>
+      <c r="B46" s="29" t="n">
+        <v>11700</v>
+      </c>
+      <c r="C46" s="29" t="n">
+        <v>34300</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="28" t="inlineStr">
+        <is>
+          <t>TOTAL OPEX (incl. payroll)</t>
+        </is>
+      </c>
+      <c r="B48" s="29" t="n">
+        <v>33200</v>
+      </c>
+      <c r="C48" s="29" t="n">
+        <v>186350</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="28" t="inlineStr">
+        <is>
+          <t>Operating Result</t>
+        </is>
+      </c>
+      <c r="B50" s="29" t="n">
+        <v>9200</v>
+      </c>
+      <c r="C50" s="29" t="n">
+        <v>-950</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="23" t="inlineStr">
+        <is>
+          <t>Cash Flow Impact (Year 3)</t>
+        </is>
+      </c>
+      <c r="B53" s="24" t="n"/>
+      <c r="C53" s="24" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Opening cash (Y3, identical in both cases — from shared Y1-Y2)</t>
+        </is>
+      </c>
+      <c r="B54" s="25" t="n">
+        <v>8220</v>
+      </c>
+      <c r="C54" s="25" t="n">
+        <v>8220</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Total receipts (= Total Revenue above)</t>
+        </is>
+      </c>
+      <c r="B55" s="25" t="n">
+        <v>48000</v>
+      </c>
+      <c r="C55" s="25" t="n">
+        <v>210000</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="28" t="inlineStr">
+        <is>
+          <t>Total expenditure (COGS + Total Employment Cost + Other OPEX + Corp tax)</t>
+        </is>
+      </c>
+      <c r="B56" s="29" t="n">
+        <v>-39800</v>
+      </c>
+      <c r="C56" s="29" t="n">
+        <v>-211450</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="28" t="inlineStr">
+        <is>
+          <t>Net cash movement in year</t>
+        </is>
+      </c>
+      <c r="B57" s="29" t="n">
+        <v>8200</v>
+      </c>
+      <c r="C57" s="29" t="n">
+        <v>-1450</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="28" t="inlineStr">
+        <is>
+          <t>Closing cash</t>
+        </is>
+      </c>
+      <c r="B58" s="29" t="n">
+        <v>16420</v>
+      </c>
+      <c r="C58" s="29" t="n">
+        <v>6770</v>
+      </c>
+    </row>
+    <row r="59" ht="60" customHeight="1">
+      <c r="A59" s="20" t="inlineStr">
+        <is>
+          <t>Reconciliation note: this upside case ends Year 3 with £6,770 of cash on the books (down from the base case's £16,420, since the extra wage bill outpaces the extra revenue slightly) but does not require any external funding — it is funded entirely by the additional institutional and premium revenue generated once 5+ universities convert post-pilot. This is an annual figure only; no month-by-month cash flow has been modelled for this scenario, so intra-year dips (e.g. before new hires' revenue impact ramps up) are not ruled out. Presented as an illustrative target, not a committed forecast — the core 3-year model (P&amp;L 3yr, Payroll W3) remains the conservative base case this business plan is built on.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A59:C59"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>